<commit_message>
fix: use correct CCDC file, update ledger files, adjust DATA_DIR
</commit_message>
<xml_diff>
--- a/Bảng cân đối số phát sinh.xlsx
+++ b/Bảng cân đối số phát sinh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://shinegroupvn-my.sharepoint.com/personal/alba_shine-group_com_vn/Documents/Desktop/Vi - Alba/Alba - CCDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_8764A6B4C34C3F735CFF2BAFAFC2139E587826A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B2B8914-E943-4E9C-9A3C-E538B8A4CC0D}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_8764A6B42E647F49A8FF2BAFAFC2136BB03A498D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{386644EB-B550-4B5B-9F61-A8032BE0057C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
     <t>BẢNG CÂN ĐỐI SỐ PHÁT SINH</t>
   </si>
   <si>
-    <t>Tháng 01 năm 2026</t>
+    <t>Sáu tháng đầu năm 2026</t>
   </si>
   <si>
     <t>SỐ HIỆU TÀI KHOẢN</t>
@@ -1050,15 +1050,15 @@
         <v>0</v>
       </c>
       <c r="F10" s="21">
-        <v>-855136923</v>
+        <v>435995043</v>
       </c>
       <c r="G10" s="27">
-        <v>-668347875</v>
+        <v>2745890919</v>
       </c>
       <c r="H10" s="27"/>
       <c r="I10" s="27"/>
       <c r="J10" s="21">
-        <v>53907663152</v>
+        <v>51784556324</v>
       </c>
       <c r="K10" s="25">
         <v>0</v>
@@ -1079,15 +1079,15 @@
         <v>0</v>
       </c>
       <c r="F11" s="22">
-        <v>-969686800</v>
+        <v>-252904749</v>
       </c>
       <c r="G11" s="29">
-        <v>139247638</v>
+        <v>861559619</v>
       </c>
       <c r="H11" s="29"/>
       <c r="I11" s="29"/>
       <c r="J11" s="22">
-        <v>276495277</v>
+        <v>270965347</v>
       </c>
       <c r="K11" s="26">
         <v>0</v>
@@ -1108,15 +1108,15 @@
         <v>0</v>
       </c>
       <c r="F12" s="22">
-        <v>114549877</v>
+        <v>688899792</v>
       </c>
       <c r="G12" s="29">
-        <v>-807595513</v>
+        <v>1884331300</v>
       </c>
       <c r="H12" s="29"/>
       <c r="I12" s="29"/>
       <c r="J12" s="22">
-        <v>53631167875</v>
+        <v>51513590977</v>
       </c>
       <c r="K12" s="26">
         <v>0</v>
@@ -1182,12 +1182,12 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="C13:G13"/>
     <mergeCell ref="H13:K13"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="G12:I12"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="G10:I10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="G11:I11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="G12:I12"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="G9:I9"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>